<commit_message>
Fixing super broken things
</commit_message>
<xml_diff>
--- a/src/server/savedSwims.xlsx
+++ b/src/server/savedSwims.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -559,9 +559,31 @@
         <v>4000</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>1782601042466</v>
+      </c>
+      <c r="B15" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C15">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>1782601044377</v>
+      </c>
+      <c r="B16" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C16">
+        <v>4000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Back and forth working
</commit_message>
<xml_diff>
--- a/src/server/savedSwims.xlsx
+++ b/src/server/savedSwims.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -581,9 +581,31 @@
         <v>4000</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>1782619519216</v>
+      </c>
+      <c r="B17" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C17">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>1782619597203</v>
+      </c>
+      <c r="B18" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C18">
+        <v>4000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Another round of tweaking the save and read
</commit_message>
<xml_diff>
--- a/src/server/savedSwims.xlsx
+++ b/src/server/savedSwims.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,199 +413,106 @@
         <v>interval</v>
       </c>
       <c r="E1" t="str">
+        <v>mainSetYardage</v>
+      </c>
+      <c r="F1" t="str">
+        <v>warmUp</v>
+      </c>
+      <c r="G1" t="str">
+        <v>coolDown</v>
+      </c>
+      <c r="H1" t="str">
+        <v>rounds</v>
+      </c>
+      <c r="I1" t="str">
+        <v>maxDistance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>intervalTime</v>
+      </c>
+      <c r="K1" t="str">
+        <v>totalDistance</v>
+      </c>
+      <c r="L1" t="str">
         <v>workoutDetails</v>
+      </c>
+      <c r="M1" t="str">
+        <v>createdAt</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1780460000101</v>
+        <v>1782621757960</v>
       </c>
       <c r="B2" t="str">
         <v>distance</v>
       </c>
       <c r="C2">
-        <v>4000</v>
+        <v>9500</v>
+      </c>
+      <c r="D2">
+        <v>90</v>
+      </c>
+      <c r="E2">
+        <v>6200</v>
+      </c>
+      <c r="F2">
+        <v>2100</v>
+      </c>
+      <c r="G2">
+        <v>1200</v>
+      </c>
+      <c r="H2">
+        <v>62</v>
+      </c>
+      <c r="I2">
+        <v>100</v>
+      </c>
+      <c r="J2">
+        <v>90</v>
+      </c>
+      <c r="K2">
+        <v>6200</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1780544903325</v>
+        <v>1782622040276</v>
       </c>
       <c r="B3" t="str">
         <v>distance</v>
       </c>
       <c r="C3">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>1780546838724</v>
-      </c>
-      <c r="B4" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C4">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>1781843360398</v>
-      </c>
-      <c r="B5" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C5">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>1782595680975</v>
-      </c>
-      <c r="B6" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C6">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>1782595811930</v>
-      </c>
-      <c r="B7" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C7">
-        <v>4100</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>1782598607541</v>
-      </c>
-      <c r="B8" t="str">
-        <v>easy</v>
-      </c>
-      <c r="C8">
-        <v>4100</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>1782600345574</v>
-      </c>
-      <c r="B9" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C9">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>1782600480156</v>
-      </c>
-      <c r="B10" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C10">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>1782600497725</v>
-      </c>
-      <c r="B11" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C11">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>1782600571760</v>
-      </c>
-      <c r="B12" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C12">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>1782600684468</v>
-      </c>
-      <c r="B13" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C13">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>1782600692373</v>
-      </c>
-      <c r="B14" t="str">
-        <v>threshold</v>
-      </c>
-      <c r="C14">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>1782601042466</v>
-      </c>
-      <c r="B15" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C15">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>1782601044377</v>
-      </c>
-      <c r="B16" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C16">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>1782619519216</v>
-      </c>
-      <c r="B17" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C17">
         <v>5000</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>1782619597203</v>
-      </c>
-      <c r="B18" t="str">
-        <v>distance</v>
-      </c>
-      <c r="C18">
-        <v>4000</v>
+      <c r="D3">
+        <v>90</v>
+      </c>
+      <c r="E3">
+        <v>3300</v>
+      </c>
+      <c r="F3">
+        <v>1100</v>
+      </c>
+      <c r="G3">
+        <v>600</v>
+      </c>
+      <c r="H3">
+        <v>33</v>
+      </c>
+      <c r="I3">
+        <v>100</v>
+      </c>
+      <c r="J3">
+        <v>90</v>
+      </c>
+      <c r="K3">
+        <v>3300</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Distance saved sets are now showing. Needs so much more work but we have a it displaying
</commit_message>
<xml_diff>
--- a/src/server/savedSwims.xlsx
+++ b/src/server/savedSwims.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -580,9 +580,35 @@
         <v>2900</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6">
+        <v>1782708742158</v>
+      </c>
+      <c r="B6" t="str">
+        <v>sprint</v>
+      </c>
+      <c r="C6">
+        <v>4000</v>
+      </c>
+      <c r="D6">
+        <v>90</v>
+      </c>
+      <c r="E6">
+        <v>2000</v>
+      </c>
+      <c r="F6">
+        <v>1300</v>
+      </c>
+      <c r="G6">
+        <v>700</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Saved workouts now formatted
</commit_message>
<xml_diff>
--- a/src/server/savedSwims.xlsx
+++ b/src/server/savedSwims.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:AA10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,6 +437,48 @@
         <v>workoutDetails</v>
       </c>
       <c r="M1" t="str">
+        <v>sprintRounds</v>
+      </c>
+      <c r="N1" t="str">
+        <v>sprintDistance</v>
+      </c>
+      <c r="O1" t="str">
+        <v>easyDistance</v>
+      </c>
+      <c r="P1" t="str">
+        <v>kickDistance</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>kickRounds</v>
+      </c>
+      <c r="R1" t="str">
+        <v>pullDistance</v>
+      </c>
+      <c r="S1" t="str">
+        <v>pullRounds</v>
+      </c>
+      <c r="T1" t="str">
+        <v>drillDistance</v>
+      </c>
+      <c r="U1" t="str">
+        <v>drillRounds</v>
+      </c>
+      <c r="V1" t="str">
+        <v>drills</v>
+      </c>
+      <c r="W1" t="str">
+        <v>breathDistance</v>
+      </c>
+      <c r="X1" t="str">
+        <v>breathRounds</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>breathWorkoutPattern</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>breathWorkPatternText</v>
+      </c>
+      <c r="AA1" t="str">
         <v>createdAt</v>
       </c>
     </row>
@@ -606,9 +648,152 @@
         <v>5</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>1782791961584</v>
+      </c>
+      <c r="B7" t="str">
+        <v>sprint</v>
+      </c>
+      <c r="C7">
+        <v>4000</v>
+      </c>
+      <c r="D7">
+        <v>90</v>
+      </c>
+      <c r="E7">
+        <v>2000</v>
+      </c>
+      <c r="F7">
+        <v>1300</v>
+      </c>
+      <c r="G7">
+        <v>700</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>1782793280478</v>
+      </c>
+      <c r="B8" t="str">
+        <v>sprint</v>
+      </c>
+      <c r="C8">
+        <v>4000</v>
+      </c>
+      <c r="D8">
+        <v>90</v>
+      </c>
+      <c r="E8">
+        <v>2000</v>
+      </c>
+      <c r="F8">
+        <v>1300</v>
+      </c>
+      <c r="G8">
+        <v>700</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+      <c r="N8">
+        <v>50</v>
+      </c>
+      <c r="O8">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1782793286711</v>
+      </c>
+      <c r="B9" t="str">
+        <v>threshold</v>
+      </c>
+      <c r="C9">
+        <v>4000</v>
+      </c>
+      <c r="D9">
+        <v>90</v>
+      </c>
+      <c r="E9">
+        <v>2000</v>
+      </c>
+      <c r="F9">
+        <v>1300</v>
+      </c>
+      <c r="G9">
+        <v>700</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>200</v>
+      </c>
+      <c r="J9">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>1782793294947</v>
+      </c>
+      <c r="B10" t="str">
+        <v>easy</v>
+      </c>
+      <c r="C10">
+        <v>4000</v>
+      </c>
+      <c r="D10">
+        <v>90</v>
+      </c>
+      <c r="E10">
+        <v>2600</v>
+      </c>
+      <c r="F10">
+        <v>900</v>
+      </c>
+      <c r="G10">
+        <v>500</v>
+      </c>
+      <c r="P10">
+        <v>200</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="R10">
+        <v>500</v>
+      </c>
+      <c r="S10">
+        <v>5</v>
+      </c>
+      <c r="T10">
+        <v>700</v>
+      </c>
+      <c r="U10">
+        <v>1</v>
+      </c>
+      <c r="W10">
+        <v>1200</v>
+      </c>
+      <c r="X10">
+        <v>2</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>[3, 5]</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>